<commit_message>
update data input for simulation Las 1B
</commit_message>
<xml_diff>
--- a/Data Input/BAU_Lahan.xlsx
+++ b/Data Input/BAU_Lahan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/dw/ICRAF/analisis data/CIFOR-ICRAF indonesia/Solusi/Jawa Tengah/0_Regional Ekonomi/R - Regional Ekonomi Jateng/Data Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{C1A1B4A4-1878-4794-BDFA-AD98FB9CBDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4FFC83A-1BFC-4C41-9808-B6D2F722042B}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{C1A1B4A4-1878-4794-BDFA-AD98FB9CBDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{082D5C4C-4788-55F2-BD74-03E4D9734450}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A483B452-8B02-4646-B940-D3630FDC5529}"/>
   </bookViews>
@@ -169,7 +169,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -194,6 +194,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -211,13 +217,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -225,6 +232,7 @@
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -401,14 +409,15 @@
   <dimension ref="A1:W26"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="2.796875" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.59765625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="15" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.69921875" style="7"/>
+    <col min="1" max="1" width="2.796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.59765625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="10" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="13.09765625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="23" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.69921875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="6" customFormat="1">
+    <row r="1" spans="1:23" s="7" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -418,16 +427,16 @@
       <c r="C1" s="2">
         <v>2025</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="2">
         <v>2026</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="2">
         <v>2027</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="2">
         <v>2028</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="2">
         <v>2029</v>
       </c>
       <c r="H1" s="3">
@@ -436,46 +445,46 @@
       <c r="I1" s="4">
         <v>2031</v>
       </c>
-      <c r="J1" s="4">
+      <c r="J1" s="5">
         <v>2032</v>
       </c>
-      <c r="K1" s="4">
+      <c r="K1" s="6">
         <v>2033</v>
       </c>
-      <c r="L1" s="4">
+      <c r="L1" s="3">
         <v>2034</v>
       </c>
-      <c r="M1" s="4">
+      <c r="M1" s="3">
         <v>2035</v>
       </c>
-      <c r="N1" s="5">
+      <c r="N1" s="3">
         <v>2036</v>
       </c>
-      <c r="O1" s="5">
+      <c r="O1" s="3">
         <v>2037</v>
       </c>
-      <c r="P1" s="6">
+      <c r="P1" s="3">
         <v>2038</v>
       </c>
-      <c r="Q1" s="6">
+      <c r="Q1" s="4">
         <v>2039</v>
       </c>
-      <c r="R1" s="6">
+      <c r="R1" s="4">
         <v>2040</v>
       </c>
-      <c r="S1" s="6">
+      <c r="S1" s="4">
         <v>2041</v>
       </c>
-      <c r="T1" s="6">
+      <c r="T1" s="4">
         <v>2042</v>
       </c>
-      <c r="U1" s="6">
+      <c r="U1" s="4">
         <v>2043</v>
       </c>
-      <c r="V1" s="6">
+      <c r="V1" s="5">
         <v>2044</v>
       </c>
-      <c r="W1" s="6">
+      <c r="W1" s="5">
         <v>2045</v>
       </c>
     </row>
@@ -486,7 +495,7 @@
       <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="10">
         <v>2693</v>
       </c>
       <c r="D2" s="10">
@@ -501,16 +510,16 @@
       <c r="G2" s="10">
         <v>2109.8699153134207</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="11">
         <v>1985.0000000000005</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2" s="12">
         <v>1960.3976629639017</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="13">
         <v>1936.1002503548248</v>
       </c>
-      <c r="K2" s="11">
+      <c r="K2" s="14">
         <v>1912.1039829014726</v>
       </c>
       <c r="L2" s="11">
@@ -519,34 +528,34 @@
       <c r="M2" s="11">
         <v>1864.9999999999993</v>
       </c>
-      <c r="N2" s="12">
+      <c r="N2" s="11">
         <v>1864.199312788385</v>
       </c>
-      <c r="O2" s="12">
+      <c r="O2" s="11">
         <v>1863.3989693301269</v>
       </c>
-      <c r="P2" s="7">
+      <c r="P2" s="11">
         <v>1862.5989694776447</v>
       </c>
-      <c r="Q2" s="7">
+      <c r="Q2" s="12">
         <v>1861.7993130834204</v>
       </c>
-      <c r="R2" s="7">
+      <c r="R2" s="12">
         <v>1860.9999999999998</v>
       </c>
-      <c r="S2" s="7">
+      <c r="S2" s="12">
         <v>1861</v>
       </c>
-      <c r="T2" s="7">
+      <c r="T2" s="12">
         <v>1861</v>
       </c>
-      <c r="U2" s="7">
+      <c r="U2" s="12">
         <v>1861</v>
       </c>
-      <c r="V2" s="7">
+      <c r="V2" s="13">
         <v>1861</v>
       </c>
-      <c r="W2" s="7">
+      <c r="W2" s="13">
         <v>1861</v>
       </c>
     </row>
@@ -557,7 +566,7 @@
       <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>14514</v>
       </c>
       <c r="D3" s="10">
@@ -572,16 +581,16 @@
       <c r="G3" s="10">
         <v>13841.256066368347</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="11">
         <v>13678.000000000002</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="12">
         <v>13492.221486074384</v>
       </c>
-      <c r="J3" s="11">
+      <c r="J3" s="13">
         <v>13308.966269139293</v>
       </c>
-      <c r="K3" s="11">
+      <c r="K3" s="14">
         <v>13128.20007705223</v>
       </c>
       <c r="L3" s="11">
@@ -590,34 +599,34 @@
       <c r="M3" s="11">
         <v>12774.000000000002</v>
       </c>
-      <c r="N3" s="12">
+      <c r="N3" s="11">
         <v>12657.701558109957</v>
       </c>
-      <c r="O3" s="12">
+      <c r="O3" s="11">
         <v>12542.461933159482</v>
       </c>
-      <c r="P3" s="7">
+      <c r="P3" s="11">
         <v>12428.27148535209</v>
       </c>
-      <c r="Q3" s="7">
+      <c r="Q3" s="12">
         <v>12315.120662654977</v>
       </c>
-      <c r="R3" s="7">
+      <c r="R3" s="12">
         <v>12203.000000000002</v>
       </c>
-      <c r="S3" s="7">
+      <c r="S3" s="12">
         <v>12122.340743276915</v>
       </c>
-      <c r="T3" s="7">
+      <c r="T3" s="12">
         <v>12042.214627231951</v>
       </c>
-      <c r="U3" s="7">
+      <c r="U3" s="12">
         <v>11962.618127917653</v>
       </c>
-      <c r="V3" s="7">
+      <c r="V3" s="13">
         <v>11883.547744679108</v>
       </c>
-      <c r="W3" s="7">
+      <c r="W3" s="13">
         <v>11805.000000000004</v>
       </c>
     </row>
@@ -628,7 +637,7 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>90</v>
       </c>
       <c r="D4" s="10">
@@ -643,16 +652,16 @@
       <c r="G4" s="10">
         <v>93.186024607269403</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="11">
         <v>94.000000000000043</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="12">
         <v>94.592483899005074</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="13">
         <v>95.188702235995052</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="14">
         <v>95.788678549207987</v>
       </c>
       <c r="L4" s="11">
@@ -661,34 +670,34 @@
       <c r="M4" s="11">
         <v>97.000000000000043</v>
       </c>
-      <c r="N4" s="12">
+      <c r="N4" s="11">
         <v>97.787121480942545</v>
       </c>
-      <c r="O4" s="12">
+      <c r="O4" s="11">
         <v>98.580630180707374</v>
       </c>
-      <c r="P4" s="7">
+      <c r="P4" s="11">
         <v>99.380577929368073</v>
       </c>
-      <c r="Q4" s="7">
+      <c r="Q4" s="12">
         <v>100.18701697758138</v>
       </c>
-      <c r="R4" s="7">
+      <c r="R4" s="12">
         <v>101.00000000000004</v>
       </c>
-      <c r="S4" s="7">
+      <c r="S4" s="12">
         <v>101.78761977456811</v>
       </c>
-      <c r="T4" s="7">
+      <c r="T4" s="12">
         <v>102.58138157794109</v>
       </c>
-      <c r="U4" s="7">
+      <c r="U4" s="12">
         <v>103.38133330698371</v>
       </c>
-      <c r="V4" s="7">
+      <c r="V4" s="13">
         <v>104.18752323207082</v>
       </c>
-      <c r="W4" s="7">
+      <c r="W4" s="13">
         <v>105.00000000000007</v>
       </c>
     </row>
@@ -699,7 +708,7 @@
       <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>6825</v>
       </c>
       <c r="D5" s="10">
@@ -714,16 +723,16 @@
       <c r="G5" s="10">
         <v>6700.7157976209428</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="11">
         <v>6670.0000000000018</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="12">
         <v>6663.788441516047</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="13">
         <v>6657.5826676586012</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="14">
         <v>6651.3826730406236</v>
       </c>
       <c r="L5" s="11">
@@ -732,34 +741,34 @@
       <c r="M5" s="11">
         <v>6638.9999999999991</v>
       </c>
-      <c r="N5" s="12">
+      <c r="N5" s="11">
         <v>6635.9972850670401</v>
       </c>
-      <c r="O5" s="12">
+      <c r="O5" s="11">
         <v>6632.9959282146601</v>
       </c>
-      <c r="P5" s="7">
+      <c r="P5" s="11">
         <v>6629.9959288286209</v>
       </c>
-      <c r="Q5" s="7">
+      <c r="Q5" s="12">
         <v>6626.9972862949626</v>
       </c>
-      <c r="R5" s="7">
+      <c r="R5" s="12">
         <v>6624.0000000000018</v>
       </c>
-      <c r="S5" s="7">
+      <c r="S5" s="12">
         <v>6620.9972789107251</v>
       </c>
-      <c r="T5" s="7">
+      <c r="T5" s="12">
         <v>6617.9959189829751</v>
       </c>
-      <c r="U5" s="7">
+      <c r="U5" s="12">
         <v>6614.9959195997226</v>
       </c>
-      <c r="V5" s="7">
+      <c r="V5" s="13">
         <v>6611.99728014422</v>
       </c>
-      <c r="W5" s="7">
+      <c r="W5" s="13">
         <v>6608.9999999999991</v>
       </c>
     </row>
@@ -770,7 +779,7 @@
       <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>298</v>
       </c>
       <c r="D6" s="10">
@@ -785,16 +794,16 @@
       <c r="G6" s="10">
         <v>312.31505443505483</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="11">
         <v>315.99999999999994</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="12">
         <v>319.52067092795841</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="13">
         <v>323.08056693117936</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="14">
         <v>326.68012503049238</v>
       </c>
       <c r="L6" s="11">
@@ -803,34 +812,34 @@
       <c r="M6" s="11">
         <v>334.00000000000011</v>
       </c>
-      <c r="N6" s="12">
+      <c r="N6" s="11">
         <v>337.33281987704913</v>
       </c>
-      <c r="O6" s="12">
+      <c r="O6" s="11">
         <v>340.69889630599306</v>
       </c>
-      <c r="P6" s="7">
+      <c r="P6" s="11">
         <v>344.09856113742217</v>
       </c>
-      <c r="Q6" s="7">
+      <c r="Q6" s="12">
         <v>347.53214953329882</v>
       </c>
-      <c r="R6" s="7">
+      <c r="R6" s="12">
         <v>351</v>
       </c>
-      <c r="S6" s="7">
+      <c r="S6" s="12">
         <v>354.14319903385723</v>
       </c>
-      <c r="T6" s="7">
+      <c r="T6" s="12">
         <v>357.31454536163596</v>
       </c>
-      <c r="U6" s="7">
+      <c r="U6" s="12">
         <v>360.5142910418748</v>
       </c>
-      <c r="V6" s="7">
+      <c r="V6" s="13">
         <v>363.7426903902923</v>
       </c>
-      <c r="W6" s="7">
+      <c r="W6" s="13">
         <v>367</v>
       </c>
     </row>
@@ -841,7 +850,7 @@
       <c r="B7" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>56897</v>
       </c>
       <c r="D7" s="10">
@@ -856,16 +865,16 @@
       <c r="G7" s="10">
         <v>51661.742228586249</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="11">
         <v>50429.999999999978</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="12">
         <v>49798.795667198297</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="13">
         <v>49175.491768855201</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="14">
         <v>48559.989419615544</v>
       </c>
       <c r="L7" s="11">
@@ -874,34 +883,34 @@
       <c r="M7" s="11">
         <v>47351.999999999993</v>
       </c>
-      <c r="N7" s="12">
+      <c r="N7" s="11">
         <v>46790.857072401581</v>
       </c>
-      <c r="O7" s="12">
+      <c r="O7" s="11">
         <v>46236.363945977209</v>
       </c>
-      <c r="P7" s="7">
+      <c r="P7" s="11">
         <v>45688.441817531697</v>
       </c>
-      <c r="Q7" s="7">
+      <c r="Q7" s="12">
         <v>45147.012817723873</v>
       </c>
-      <c r="R7" s="7">
+      <c r="R7" s="12">
         <v>44611.999999999993</v>
       </c>
-      <c r="S7" s="7">
+      <c r="S7" s="12">
         <v>43979.942098996398</v>
       </c>
-      <c r="T7" s="7">
+      <c r="T7" s="12">
         <v>43356.839124699087</v>
       </c>
-      <c r="U7" s="7">
+      <c r="U7" s="12">
         <v>42742.564204693081</v>
       </c>
-      <c r="V7" s="7">
+      <c r="V7" s="13">
         <v>42136.99226407778</v>
       </c>
-      <c r="W7" s="7">
+      <c r="W7" s="13">
         <v>41540</v>
       </c>
     </row>
@@ -912,7 +921,7 @@
       <c r="B8" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="10">
         <v>43964</v>
       </c>
       <c r="D8" s="10">
@@ -927,16 +936,16 @@
       <c r="G8" s="10">
         <v>43573.164720480621</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="11">
         <v>43476.000000000007</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="12">
         <v>43422.669322178175</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="13">
         <v>43369.40406346567</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="14">
         <v>43316.204143614872</v>
       </c>
       <c r="L8" s="11">
@@ -945,34 +954,34 @@
       <c r="M8" s="11">
         <v>43209.999999999985</v>
       </c>
-      <c r="N8" s="12">
+      <c r="N8" s="11">
         <v>43149.832674390273</v>
       </c>
-      <c r="O8" s="12">
+      <c r="O8" s="11">
         <v>43089.749128161959</v>
       </c>
-      <c r="P8" s="7">
+      <c r="P8" s="11">
         <v>43029.749244657316</v>
       </c>
-      <c r="Q8" s="7">
+      <c r="Q8" s="12">
         <v>42969.832907381031</v>
       </c>
-      <c r="R8" s="7">
+      <c r="R8" s="12">
         <v>42910.000000000007</v>
       </c>
-      <c r="S8" s="7">
+      <c r="S8" s="12">
         <v>42839.166529716611</v>
       </c>
-      <c r="T8" s="7">
+      <c r="T8" s="12">
         <v>42768.449987433974</v>
       </c>
-      <c r="U8" s="7">
+      <c r="U8" s="12">
         <v>42697.850180133777</v>
       </c>
-      <c r="V8" s="7">
+      <c r="V8" s="13">
         <v>42627.366915116319</v>
       </c>
-      <c r="W8" s="7">
+      <c r="W8" s="13">
         <v>42557.000000000007</v>
       </c>
     </row>
@@ -983,7 +992,7 @@
       <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
         <v>9317</v>
       </c>
       <c r="D9" s="10">
@@ -998,16 +1007,16 @@
       <c r="G9" s="10">
         <v>9132.5412294668349</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="11">
         <v>9087</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="12">
         <v>9076.9779175924068</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="13">
         <v>9066.9668885727078</v>
       </c>
-      <c r="K9" s="11">
+      <c r="K9" s="14">
         <v>9056.9669007500834</v>
       </c>
       <c r="L9" s="11">
@@ -1016,34 +1025,34 @@
       <c r="M9" s="11">
         <v>9036.9999999999982</v>
       </c>
-      <c r="N9" s="12">
+      <c r="N9" s="11">
         <v>9035.7996811831563</v>
       </c>
-      <c r="O9" s="12">
+      <c r="O9" s="11">
         <v>9034.599521795908</v>
       </c>
-      <c r="P9" s="7">
+      <c r="P9" s="11">
         <v>9033.3995218170803</v>
       </c>
-      <c r="Q9" s="7">
+      <c r="Q9" s="12">
         <v>9032.1996812255002</v>
       </c>
-      <c r="R9" s="7">
+      <c r="R9" s="12">
         <v>9030.9999999999982</v>
       </c>
-      <c r="S9" s="7">
+      <c r="S9" s="12">
         <v>9029.1992820421474</v>
       </c>
-      <c r="T9" s="7">
+      <c r="T9" s="12">
         <v>9027.398923134806</v>
       </c>
-      <c r="U9" s="7">
+      <c r="U9" s="12">
         <v>9025.5989232063839</v>
       </c>
-      <c r="V9" s="7">
+      <c r="V9" s="13">
         <v>9023.7992821853022</v>
       </c>
-      <c r="W9" s="7">
+      <c r="W9" s="13">
         <v>9021.9999999999982</v>
       </c>
     </row>
@@ -1054,7 +1063,7 @@
       <c r="B10" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <v>8534</v>
       </c>
       <c r="D10" s="10">
@@ -1069,16 +1078,16 @@
       <c r="G10" s="10">
         <v>9127.3305500894057</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="11">
         <v>9282.0000000000036</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="12">
         <v>9287.1941834424615</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="13">
         <v>9292.3912735366812</v>
       </c>
-      <c r="K10" s="11">
+      <c r="K10" s="14">
         <v>9297.5912719092157</v>
       </c>
       <c r="L10" s="11">
@@ -1087,34 +1096,34 @@
       <c r="M10" s="11">
         <v>9308.0000000000018</v>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="11">
         <v>9286.2990471225894</v>
       </c>
-      <c r="O10" s="12">
+      <c r="O10" s="11">
         <v>9264.6486885034283</v>
       </c>
-      <c r="P10" s="7">
+      <c r="P10" s="11">
         <v>9243.0488061855322</v>
       </c>
-      <c r="Q10" s="7">
+      <c r="Q10" s="12">
         <v>9221.4992824869241</v>
       </c>
-      <c r="R10" s="7">
+      <c r="R10" s="12">
         <v>9199.9999999999964</v>
       </c>
-      <c r="S10" s="7">
+      <c r="S10" s="12">
         <v>9221.4992824869259</v>
       </c>
-      <c r="T10" s="7">
+      <c r="T10" s="12">
         <v>9243.0488061855322</v>
       </c>
-      <c r="U10" s="7">
+      <c r="U10" s="12">
         <v>9264.6486885034265</v>
       </c>
-      <c r="V10" s="7">
+      <c r="V10" s="13">
         <v>9286.2990471225858</v>
       </c>
-      <c r="W10" s="7">
+      <c r="W10" s="13">
         <v>9307.9999999999945</v>
       </c>
     </row>
@@ -1125,7 +1134,7 @@
       <c r="B11" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>2620</v>
       </c>
       <c r="D11" s="10">
@@ -1140,16 +1149,16 @@
       <c r="G11" s="10">
         <v>2678.2390686314834</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="11">
         <v>2693.0000000000005</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="12">
         <v>2704.6979299856093</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="13">
         <v>2716.446673772165</v>
       </c>
-      <c r="K11" s="11">
+      <c r="K11" s="14">
         <v>2728.2464520861004</v>
       </c>
       <c r="L11" s="11">
@@ -1158,34 +1167,34 @@
       <c r="M11" s="11">
         <v>2751.9999999999991</v>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="11">
         <v>2764.6825650938072</v>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="11">
         <v>2777.423577664852</v>
       </c>
-      <c r="P11" s="7">
+      <c r="P11" s="11">
         <v>2790.2233070677621</v>
       </c>
-      <c r="Q11" s="7">
+      <c r="Q11" s="12">
         <v>2803.0820238984829</v>
       </c>
-      <c r="R11" s="7">
+      <c r="R11" s="12">
         <v>2815.9999999999991</v>
       </c>
-      <c r="S11" s="7">
+      <c r="S11" s="12">
         <v>2827.7023331816044</v>
       </c>
-      <c r="T11" s="7">
+      <c r="T11" s="12">
         <v>2839.4532972587676</v>
       </c>
-      <c r="U11" s="7">
+      <c r="U11" s="12">
         <v>2851.2530943248639</v>
       </c>
-      <c r="V11" s="7">
+      <c r="V11" s="13">
         <v>2863.1019273130992</v>
       </c>
-      <c r="W11" s="7">
+      <c r="W11" s="13">
         <v>2874.9999999999995</v>
       </c>
     </row>
@@ -1196,7 +1205,7 @@
       <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>109817</v>
       </c>
       <c r="D12" s="10">
@@ -1211,16 +1220,16 @@
       <c r="G12" s="10">
         <v>106480.22902592787</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="11">
         <v>105661.99999999996</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="12">
         <v>104925.60695855004</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="13">
         <v>104194.34608108993</v>
       </c>
-      <c r="K12" s="11">
+      <c r="K12" s="14">
         <v>103468.18159989003</v>
       </c>
       <c r="L12" s="11">
@@ -1229,34 +1238,34 @@
       <c r="M12" s="11">
         <v>102031.00000000001</v>
       </c>
-      <c r="N12" s="12">
+      <c r="N12" s="11">
         <v>101622.3395037204</v>
       </c>
-      <c r="O12" s="12">
+      <c r="O12" s="11">
         <v>101215.31579823204</v>
       </c>
-      <c r="P12" s="7">
+      <c r="P12" s="11">
         <v>100809.92232776521</v>
       </c>
-      <c r="Q12" s="7">
+      <c r="Q12" s="12">
         <v>100406.15256280778</v>
       </c>
-      <c r="R12" s="7">
+      <c r="R12" s="12">
         <v>100003.99999999999</v>
       </c>
-      <c r="S12" s="7">
+      <c r="S12" s="12">
         <v>99976.584973047226</v>
       </c>
-      <c r="T12" s="7">
+      <c r="T12" s="12">
         <v>99949.177461630854</v>
       </c>
-      <c r="U12" s="7">
+      <c r="U12" s="12">
         <v>99921.777463690581</v>
       </c>
-      <c r="V12" s="7">
+      <c r="V12" s="13">
         <v>99894.384977166686</v>
       </c>
-      <c r="W12" s="7">
+      <c r="W12" s="13">
         <v>99866.999999999971</v>
       </c>
     </row>
@@ -1267,7 +1276,7 @@
       <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>1410</v>
       </c>
       <c r="D13" s="10">
@@ -1282,16 +1291,16 @@
       <c r="G13" s="10">
         <v>1315.5962970872276</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="11">
         <v>1293</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="12">
         <v>1304.9760847305895</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="13">
         <v>1317.0630949101151</v>
       </c>
-      <c r="K13" s="11">
+      <c r="K13" s="14">
         <v>1329.2620579574284</v>
       </c>
       <c r="L13" s="11">
@@ -1300,34 +1309,34 @@
       <c r="M13" s="11">
         <v>1353.9999999999995</v>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="11">
         <v>1362.6877937794593</v>
       </c>
-      <c r="O13" s="12">
+      <c r="O13" s="11">
         <v>1371.43133184308</v>
       </c>
-      <c r="P13" s="7">
+      <c r="P13" s="11">
         <v>1380.2309718680001</v>
       </c>
-      <c r="Q13" s="7">
+      <c r="Q13" s="12">
         <v>1389.0870738263545</v>
       </c>
-      <c r="R13" s="7">
+      <c r="R13" s="12">
         <v>1398</v>
       </c>
-      <c r="S13" s="7">
+      <c r="S13" s="12">
         <v>1412.8798578596807</v>
       </c>
-      <c r="T13" s="7">
+      <c r="T13" s="12">
         <v>1427.9180920926976</v>
       </c>
-      <c r="U13" s="7">
+      <c r="U13" s="12">
         <v>1443.1163884057203</v>
       </c>
-      <c r="V13" s="7">
+      <c r="V13" s="13">
         <v>1458.476450447532</v>
       </c>
-      <c r="W13" s="7">
+      <c r="W13" s="13">
         <v>1474.0000000000002</v>
       </c>
     </row>
@@ -1338,7 +1347,7 @@
       <c r="B14" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>831</v>
       </c>
       <c r="D14" s="10">
@@ -1353,16 +1362,16 @@
       <c r="G14" s="10">
         <v>850.94054382284071</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="11">
         <v>856</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="12">
         <v>859.5700961331363</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="13">
         <v>863.15508197001077</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="14">
         <v>866.7550196107095</v>
       </c>
       <c r="L14" s="11">
@@ -1371,34 +1380,34 @@
       <c r="M14" s="11">
         <v>874.00000000000023</v>
       </c>
-      <c r="N14" s="12">
+      <c r="N14" s="11">
         <v>877.3738514888048</v>
       </c>
-      <c r="O14" s="12">
+      <c r="O14" s="11">
         <v>880.7607268607544</v>
       </c>
-      <c r="P14" s="7">
+      <c r="P14" s="11">
         <v>884.16067639118921</v>
       </c>
-      <c r="Q14" s="7">
+      <c r="Q14" s="12">
         <v>887.57375054952456</v>
       </c>
-      <c r="R14" s="7">
+      <c r="R14" s="12">
         <v>891.00000000000011</v>
       </c>
-      <c r="S14" s="7">
+      <c r="S14" s="12">
         <v>896.92078688833328</v>
       </c>
-      <c r="T14" s="7">
+      <c r="T14" s="12">
         <v>902.88091801614701</v>
       </c>
-      <c r="U14" s="7">
+      <c r="U14" s="12">
         <v>908.88065482997013</v>
       </c>
-      <c r="V14" s="7">
+      <c r="V14" s="13">
         <v>914.92026051367054</v>
       </c>
-      <c r="W14" s="7">
+      <c r="W14" s="13">
         <v>921.00000000000034</v>
       </c>
     </row>
@@ -1409,7 +1418,7 @@
       <c r="B15" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="10">
         <v>1994</v>
       </c>
       <c r="D15" s="10">
@@ -1424,16 +1433,16 @@
       <c r="G15" s="10">
         <v>1985.995979893404</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="11">
         <v>1983.9999999999998</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="12">
         <v>1984.3998388071632</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="13">
         <v>1984.7997581945035</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K15" s="14">
         <v>1985.1997581782607</v>
       </c>
       <c r="L15" s="11">
@@ -1442,34 +1451,34 @@
       <c r="M15" s="11">
         <v>1985.9999999999993</v>
       </c>
-      <c r="N15" s="12">
+      <c r="N15" s="11">
         <v>1987.198552472069</v>
       </c>
-      <c r="O15" s="12">
+      <c r="O15" s="11">
         <v>1988.3978282714434</v>
       </c>
-      <c r="P15" s="7">
+      <c r="P15" s="11">
         <v>1989.5978278346515</v>
       </c>
-      <c r="Q15" s="7">
+      <c r="Q15" s="12">
         <v>1990.7985515984856</v>
       </c>
-      <c r="R15" s="7">
+      <c r="R15" s="12">
         <v>1992.0000000000011</v>
       </c>
-      <c r="S15" s="7">
+      <c r="S15" s="12">
         <v>1993.7967557785641</v>
       </c>
-      <c r="T15" s="7">
+      <c r="T15" s="12">
         <v>1995.5951322053852</v>
       </c>
-      <c r="U15" s="7">
+      <c r="U15" s="12">
         <v>1997.3951307422649</v>
       </c>
-      <c r="V15" s="7">
+      <c r="V15" s="13">
         <v>1999.1967528523235</v>
       </c>
-      <c r="W15" s="7">
+      <c r="W15" s="13">
         <v>2001.0000000000011</v>
       </c>
     </row>
@@ -1480,7 +1489,7 @@
       <c r="B16" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="10">
         <v>14281</v>
       </c>
       <c r="D16" s="10">
@@ -1495,16 +1504,16 @@
       <c r="G16" s="10">
         <v>14545.191874446413</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="11">
         <v>14612.000000000002</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="12">
         <v>14622.784070348367</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="13">
         <v>14633.576099646452</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16" s="14">
         <v>14644.376093768185</v>
       </c>
       <c r="L16" s="11">
@@ -1513,34 +1522,34 @@
       <c r="M16" s="11">
         <v>14665.999999999998</v>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="11">
         <v>14657.389896307664</v>
       </c>
-      <c r="O16" s="12">
+      <c r="O16" s="11">
         <v>14648.784847428202</v>
       </c>
-      <c r="P16" s="7">
+      <c r="P16" s="11">
         <v>14640.184850394036</v>
       </c>
-      <c r="Q16" s="7">
+      <c r="Q16" s="12">
         <v>14631.589902239335</v>
       </c>
-      <c r="R16" s="7">
+      <c r="R16" s="12">
         <v>14623.000000000005</v>
       </c>
-      <c r="S16" s="7">
+      <c r="S16" s="12">
         <v>14609.976823889008</v>
       </c>
-      <c r="T16" s="7">
+      <c r="T16" s="12">
         <v>14596.965246158377</v>
       </c>
-      <c r="U16" s="7">
+      <c r="U16" s="12">
         <v>14583.965256478643</v>
       </c>
-      <c r="V16" s="7">
+      <c r="V16" s="13">
         <v>14570.976844529541</v>
       </c>
-      <c r="W16" s="7">
+      <c r="W16" s="13">
         <v>14558</v>
       </c>
     </row>
@@ -1551,7 +1560,7 @@
       <c r="B17" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <v>185</v>
       </c>
       <c r="D17" s="10">
@@ -1566,16 +1575,16 @@
       <c r="G17" s="10">
         <v>210.18520021400613</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="11">
         <v>216.99999999999991</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="12">
         <v>219.73041859210244</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="13">
         <v>222.49519287862009</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17" s="14">
         <v>225.29475514262563</v>
       </c>
       <c r="L17" s="11">
@@ -1584,34 +1593,34 @@
       <c r="M17" s="11">
         <v>230.99999999999991</v>
       </c>
-      <c r="N17" s="12">
+      <c r="N17" s="11">
         <v>235.42703182657698</v>
       </c>
-      <c r="O17" s="12">
+      <c r="O17" s="11">
         <v>239.93890612412159</v>
       </c>
-      <c r="P17" s="7">
+      <c r="P17" s="11">
         <v>244.53724886804173</v>
       </c>
-      <c r="Q17" s="7">
+      <c r="Q17" s="12">
         <v>249.22371719497849</v>
       </c>
-      <c r="R17" s="7">
+      <c r="R17" s="12">
         <v>254.00000000000009</v>
       </c>
-      <c r="S17" s="7">
+      <c r="S17" s="12">
         <v>256.16285096489446</v>
       </c>
-      <c r="T17" s="7">
+      <c r="T17" s="12">
         <v>258.34411895457771</v>
       </c>
-      <c r="U17" s="7">
+      <c r="U17" s="12">
         <v>260.54396079298607</v>
       </c>
-      <c r="V17" s="7">
+      <c r="V17" s="13">
         <v>262.76253463943704</v>
       </c>
-      <c r="W17" s="7">
+      <c r="W17" s="13">
         <v>265.00000000000011</v>
       </c>
     </row>
@@ -1622,7 +1631,7 @@
       <c r="B18" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>910</v>
       </c>
       <c r="D18" s="10">
@@ -1637,16 +1646,16 @@
       <c r="G18" s="10">
         <v>1232.049801870668</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="11">
         <v>1328.9999999999993</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="12">
         <v>1388.4399005509431</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="13">
         <v>1450.5382674506493</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18" s="14">
         <v>1515.4140013578005</v>
       </c>
       <c r="L18" s="11">
@@ -1655,34 +1664,34 @@
       <c r="M18" s="11">
         <v>1654</v>
       </c>
-      <c r="N18" s="12">
+      <c r="N18" s="11">
         <v>1694.3796705433936</v>
       </c>
-      <c r="O18" s="12">
+      <c r="O18" s="11">
         <v>1735.7451438638084</v>
       </c>
-      <c r="P18" s="7">
+      <c r="P18" s="11">
         <v>1778.1204867032982</v>
       </c>
-      <c r="Q18" s="7">
+      <c r="Q18" s="12">
         <v>1821.530353353563</v>
       </c>
-      <c r="R18" s="7">
+      <c r="R18" s="12">
         <v>1866.0000000000009</v>
       </c>
-      <c r="S18" s="7">
+      <c r="S18" s="12">
         <v>1900.3145334801177</v>
       </c>
-      <c r="T18" s="7">
+      <c r="T18" s="12">
         <v>1935.2600890438141</v>
       </c>
-      <c r="U18" s="7">
+      <c r="U18" s="12">
         <v>1970.8482707791995</v>
       </c>
-      <c r="V18" s="7">
+      <c r="V18" s="13">
         <v>2007.0908961660616</v>
       </c>
-      <c r="W18" s="7">
+      <c r="W18" s="13">
         <v>2044.0000000000002</v>
       </c>
     </row>
@@ -1693,7 +1702,7 @@
       <c r="B19" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>145632</v>
       </c>
       <c r="D19" s="10">
@@ -1708,16 +1717,16 @@
       <c r="G19" s="10">
         <v>147036.71040474894</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="11">
         <v>147390.00000000009</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I19" s="12">
         <v>147266.99486203693</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="13">
         <v>147144.09237869064</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19" s="14">
         <v>147021.29246429013</v>
       </c>
       <c r="L19" s="11">
@@ -1726,34 +1735,34 @@
       <c r="M19" s="11">
         <v>146776</v>
       </c>
-      <c r="N19" s="12">
+      <c r="N19" s="11">
         <v>146382.49569059227</v>
       </c>
-      <c r="O19" s="12">
+      <c r="O19" s="11">
         <v>145990.0463604831</v>
       </c>
-      <c r="P19" s="7">
+      <c r="P19" s="11">
         <v>145598.64918128838</v>
       </c>
-      <c r="Q19" s="7">
+      <c r="Q19" s="12">
         <v>145208.30133220693</v>
       </c>
-      <c r="R19" s="7">
+      <c r="R19" s="12">
         <v>144819.00000000003</v>
       </c>
-      <c r="S19" s="7">
+      <c r="S19" s="12">
         <v>144163.08530758915</v>
       </c>
-      <c r="T19" s="7">
+      <c r="T19" s="12">
         <v>143510.14138616636</v>
       </c>
-      <c r="U19" s="7">
+      <c r="U19" s="12">
         <v>142860.15478050587</v>
       </c>
-      <c r="V19" s="7">
+      <c r="V19" s="13">
         <v>142213.11209632337</v>
       </c>
-      <c r="W19" s="7">
+      <c r="W19" s="13">
         <v>141569.00000000003</v>
       </c>
     </row>
@@ -1764,7 +1773,7 @@
       <c r="B20" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>19986</v>
       </c>
       <c r="D20" s="10">
@@ -1779,16 +1788,16 @@
       <c r="G20" s="10">
         <v>22311.513065004121</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="11">
         <v>22933.999999999996</v>
       </c>
-      <c r="I20" s="11">
+      <c r="I20" s="12">
         <v>23155.288213987638</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20" s="13">
         <v>23378.711619117243</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20" s="14">
         <v>23604.290817666406</v>
       </c>
       <c r="L20" s="11">
@@ -1797,34 +1806,34 @@
       <c r="M20" s="11">
         <v>24062.000000000004</v>
       </c>
-      <c r="N20" s="12">
+      <c r="N20" s="11">
         <v>24239.754263453644</v>
       </c>
-      <c r="O20" s="12">
+      <c r="O20" s="11">
         <v>24418.821658740715</v>
       </c>
-      <c r="P20" s="7">
+      <c r="P20" s="11">
         <v>24599.211886417354</v>
       </c>
-      <c r="Q20" s="7">
+      <c r="Q20" s="12">
         <v>24780.934718701046</v>
       </c>
-      <c r="R20" s="7">
+      <c r="R20" s="12">
         <v>24964.000000000004</v>
       </c>
-      <c r="S20" s="7">
+      <c r="S20" s="12">
         <v>25076.972860480095</v>
       </c>
-      <c r="T20" s="7">
+      <c r="T20" s="12">
         <v>25190.456971849671</v>
       </c>
-      <c r="U20" s="7">
+      <c r="U20" s="12">
         <v>25304.454647739374</v>
       </c>
-      <c r="V20" s="7">
+      <c r="V20" s="13">
         <v>25418.968212250027</v>
       </c>
-      <c r="W20" s="7">
+      <c r="W20" s="13">
         <v>25534.000000000007</v>
       </c>
     </row>
@@ -1835,7 +1844,7 @@
       <c r="B21" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="10">
         <v>2610</v>
       </c>
       <c r="D21" s="10">
@@ -1850,16 +1859,16 @@
       <c r="G21" s="10">
         <v>2472.2793519277125</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="11">
         <v>2438.9999999999991</v>
       </c>
-      <c r="I21" s="11">
+      <c r="I21" s="12">
         <v>2420.9343507839803</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21" s="13">
         <v>2403.0025136555359</v>
       </c>
-      <c r="K21" s="11">
+      <c r="K21" s="14">
         <v>2385.203497469839</v>
       </c>
       <c r="L21" s="11">
@@ -1868,34 +1877,34 @@
       <c r="M21" s="11">
         <v>2349.9999999999995</v>
       </c>
-      <c r="N21" s="12">
+      <c r="N21" s="11">
         <v>2341.1333433778232</v>
       </c>
-      <c r="O21" s="12">
+      <c r="O21" s="11">
         <v>2332.300141053372</v>
       </c>
-      <c r="P21" s="7">
+      <c r="P21" s="11">
         <v>2323.5002668020634</v>
       </c>
-      <c r="Q21" s="7">
+      <c r="Q21" s="12">
         <v>2314.7335948755654</v>
       </c>
-      <c r="R21" s="7">
+      <c r="R21" s="12">
         <v>2306</v>
       </c>
-      <c r="S21" s="7">
+      <c r="S21" s="12">
         <v>2308.395019877828</v>
       </c>
-      <c r="T21" s="7">
+      <c r="T21" s="12">
         <v>2310.7925272318985</v>
       </c>
-      <c r="U21" s="7">
+      <c r="U21" s="12">
         <v>2313.1925246457131</v>
       </c>
-      <c r="V21" s="7">
+      <c r="V21" s="13">
         <v>2315.5950147054568</v>
       </c>
-      <c r="W21" s="7">
+      <c r="W21" s="13">
         <v>2318.0000000000009</v>
       </c>
     </row>
@@ -1906,7 +1915,7 @@
       <c r="B22" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="10">
         <v>46589</v>
       </c>
       <c r="D22" s="10">
@@ -1921,16 +1930,16 @@
       <c r="G22" s="10">
         <v>51805.148368387556</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="11">
         <v>53197.999999999985</v>
       </c>
-      <c r="I22" s="11">
+      <c r="I22" s="12">
         <v>54476.275637767598</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22" s="13">
         <v>55785.266501786376</v>
       </c>
-      <c r="K22" s="11">
+      <c r="K22" s="14">
         <v>57125.710637197604</v>
       </c>
       <c r="L22" s="11">
@@ -1939,34 +1948,34 @@
       <c r="M22" s="11">
         <v>59904.000000000022</v>
       </c>
-      <c r="N22" s="12">
+      <c r="N22" s="11">
         <v>61098.965134381608</v>
       </c>
-      <c r="O22" s="12">
+      <c r="O22" s="11">
         <v>62317.767436104084</v>
       </c>
-      <c r="P22" s="7">
+      <c r="P22" s="11">
         <v>63560.882409038211</v>
       </c>
-      <c r="Q22" s="7">
+      <c r="Q22" s="12">
         <v>64828.795042407095</v>
       </c>
-      <c r="R22" s="7">
+      <c r="R22" s="12">
         <v>66122.000000000044</v>
       </c>
-      <c r="S22" s="7">
+      <c r="S22" s="12">
         <v>67266.115476908715</v>
       </c>
-      <c r="T22" s="7">
+      <c r="T22" s="12">
         <v>68430.027696573277</v>
       </c>
-      <c r="U22" s="7">
+      <c r="U22" s="12">
         <v>69614.079203982939</v>
       </c>
-      <c r="V22" s="7">
+      <c r="V22" s="13">
         <v>70818.618471216629</v>
       </c>
-      <c r="W22" s="7">
+      <c r="W22" s="13">
         <v>72043.999999999971</v>
       </c>
     </row>
@@ -1977,7 +1986,7 @@
       <c r="B23" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="10">
         <v>1622</v>
       </c>
       <c r="D23" s="10">
@@ -1992,16 +2001,16 @@
       <c r="G23" s="10">
         <v>1884.1056431270931</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="11">
         <v>1955.9999999999991</v>
       </c>
-      <c r="I23" s="11">
+      <c r="I23" s="12">
         <v>2018.302621914027</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23" s="13">
         <v>2082.5897104422475</v>
       </c>
-      <c r="K23" s="11">
+      <c r="K23" s="14">
         <v>2148.92447492677</v>
       </c>
       <c r="L23" s="11">
@@ -2010,34 +2019,34 @@
       <c r="M23" s="11">
         <v>2288</v>
       </c>
-      <c r="N23" s="12">
+      <c r="N23" s="11">
         <v>2340.1663585909264</v>
       </c>
-      <c r="O23" s="12">
+      <c r="O23" s="11">
         <v>2393.5221092135998</v>
       </c>
-      <c r="P23" s="7">
+      <c r="P23" s="11">
         <v>2448.0943699848181</v>
       </c>
-      <c r="Q23" s="7">
+      <c r="Q23" s="12">
         <v>2503.910877313951</v>
       </c>
-      <c r="R23" s="7">
+      <c r="R23" s="12">
         <v>2561.0000000000005</v>
       </c>
-      <c r="S23" s="7">
+      <c r="S23" s="12">
         <v>2613.9635656350183</v>
       </c>
-      <c r="T23" s="7">
+      <c r="T23" s="12">
         <v>2668.0224609399993</v>
       </c>
-      <c r="U23" s="7">
+      <c r="U23" s="12">
         <v>2723.1993382245359</v>
       </c>
-      <c r="V23" s="7">
+      <c r="V23" s="13">
         <v>2779.5173182664312</v>
       </c>
-      <c r="W23" s="7">
+      <c r="W23" s="13">
         <v>2837.0000000000014</v>
       </c>
     </row>
@@ -2048,7 +2057,7 @@
       <c r="B24" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="10">
         <v>2557</v>
       </c>
       <c r="D24" s="10">
@@ -2063,16 +2072,16 @@
       <c r="G24" s="10">
         <v>2604.0920837330459</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="11">
         <v>2615.9999999999995</v>
       </c>
-      <c r="I24" s="11">
+      <c r="I24" s="12">
         <v>2628.2840908732564</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24" s="13">
         <v>2640.6258648078979</v>
       </c>
-      <c r="K24" s="11">
+      <c r="K24" s="14">
         <v>2653.0255926693549</v>
       </c>
       <c r="L24" s="11">
@@ -2081,34 +2090,34 @@
       <c r="M24" s="11">
         <v>2678.0000000000005</v>
       </c>
-      <c r="N24" s="12">
+      <c r="N24" s="11">
         <v>2689.69736569834</v>
       </c>
-      <c r="O24" s="12">
+      <c r="O24" s="11">
         <v>2701.445824885956</v>
       </c>
-      <c r="P24" s="7">
+      <c r="P24" s="11">
         <v>2713.2456007365704</v>
       </c>
-      <c r="Q24" s="7">
+      <c r="Q24" s="12">
         <v>2725.0969173987169</v>
       </c>
-      <c r="R24" s="7">
+      <c r="R24" s="12">
         <v>2736.9999999999986</v>
       </c>
-      <c r="S24" s="7">
+      <c r="S24" s="12">
         <v>2746.7305654927</v>
       </c>
-      <c r="T24" s="7">
+      <c r="T24" s="12">
         <v>2756.4957250317307</v>
       </c>
-      <c r="U24" s="7">
+      <c r="U24" s="12">
         <v>2766.2956016056319</v>
       </c>
-      <c r="V24" s="7">
+      <c r="V24" s="13">
         <v>2776.1303186401919</v>
       </c>
-      <c r="W24" s="7">
+      <c r="W24" s="13">
         <v>2786.0000000000014</v>
       </c>
     </row>
@@ -2119,7 +2128,7 @@
       <c r="B25" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="10">
         <v>8989</v>
       </c>
       <c r="D25" s="10">
@@ -2134,16 +2143,16 @@
       <c r="G25" s="10">
         <v>8972.1960715306777</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="11">
         <v>8967.9999999999982</v>
       </c>
-      <c r="I25" s="11">
+      <c r="I25" s="12">
         <v>8962.9944152771823</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25" s="13">
         <v>8957.9916244747947</v>
       </c>
-      <c r="K25" s="11">
+      <c r="K25" s="14">
         <v>8952.9916260333812</v>
       </c>
       <c r="L25" s="11">
@@ -2152,34 +2161,34 @@
       <c r="M25" s="11">
         <v>8943</v>
       </c>
-      <c r="N25" s="12">
+      <c r="N25" s="11">
         <v>8938.1948390542784</v>
       </c>
-      <c r="O25" s="12">
+      <c r="O25" s="11">
         <v>8933.3922599683028</v>
       </c>
-      <c r="P25" s="7">
+      <c r="P25" s="11">
         <v>8928.5922613548155</v>
       </c>
-      <c r="Q25" s="7">
+      <c r="Q25" s="12">
         <v>8923.7948418273027</v>
       </c>
-      <c r="R25" s="7">
+      <c r="R25" s="12">
         <v>8918.9999999999982</v>
       </c>
-      <c r="S25" s="7">
+      <c r="S25" s="12">
         <v>8914.7960388022366</v>
       </c>
-      <c r="T25" s="7">
+      <c r="T25" s="12">
         <v>8910.5940591371273</v>
       </c>
-      <c r="U25" s="7">
+      <c r="U25" s="12">
         <v>8906.394060070681</v>
       </c>
-      <c r="V25" s="7">
+      <c r="V25" s="13">
         <v>8902.1960406693433</v>
       </c>
-      <c r="W25" s="7">
+      <c r="W25" s="13">
         <v>8898.0000000000018</v>
       </c>
     </row>
@@ -2190,7 +2199,7 @@
       <c r="B26" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>188</v>
       </c>
       <c r="D26" s="10">
@@ -2205,16 +2214,16 @@
       <c r="G26" s="10">
         <v>188</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="11">
         <v>188</v>
       </c>
-      <c r="I26" s="11">
+      <c r="I26" s="12">
         <v>188</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26" s="13">
         <v>188</v>
       </c>
-      <c r="K26" s="11">
+      <c r="K26" s="14">
         <v>188</v>
       </c>
       <c r="L26" s="11">
@@ -2223,44 +2232,38 @@
       <c r="M26" s="11">
         <v>188</v>
       </c>
-      <c r="N26" s="12">
+      <c r="N26" s="11">
         <v>188</v>
       </c>
-      <c r="O26" s="12">
+      <c r="O26" s="11">
         <v>188</v>
       </c>
-      <c r="P26" s="7">
+      <c r="P26" s="11">
         <v>188</v>
       </c>
-      <c r="Q26" s="7">
+      <c r="Q26" s="12">
         <v>188</v>
       </c>
-      <c r="R26" s="7">
+      <c r="R26" s="12">
         <v>188</v>
       </c>
-      <c r="S26" s="7">
+      <c r="S26" s="12">
         <v>188</v>
       </c>
-      <c r="T26" s="7">
+      <c r="T26" s="12">
         <v>188</v>
       </c>
-      <c r="U26" s="7">
+      <c r="U26" s="12">
         <v>188</v>
       </c>
-      <c r="V26" s="7">
+      <c r="V26" s="13">
         <v>188</v>
       </c>
-      <c r="W26" s="7">
+      <c r="W26" s="13">
         <v>188</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{747e98d3-0e70-4db5-a56b-cae542e688be}" enabled="0" method="" siteId="{747e98d3-0e70-4db5-a56b-cae542e688be}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>